<commit_message>
Eliminar ceros adelante en codigo principal de productos y optimizar a 1 sola pestana limpia evitando sobrecosto de memoria PHP
</commit_message>
<xml_diff>
--- a/Adaptador Convert  ecuafact zifat/Productos_Zifact_Migrado.xlsx
+++ b/Adaptador Convert  ecuafact zifat/Productos_Zifact_Migrado.xlsx
@@ -4,7 +4,6 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
-    <sheet name="Plantilla" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -459,67 +458,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Nombre</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Código Principal</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Código Auxiliar</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Precio Unitario</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Código IVA</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Código ICE</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Código IRBPNR</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Estado (A/I)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Cacao</v>
-      </c>
-      <c r="B2" t="str">
-        <v>1</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2">
-        <v>50</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="str">
-        <v>A</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Homologacion oficial Zifact de Productos usando plantilla oficial con hoja Plantilla y headers Codigo Principal sin tildes
</commit_message>
<xml_diff>
--- a/Adaptador Convert  ecuafact zifat/Productos_Zifact_Migrado.xlsx
+++ b/Adaptador Convert  ecuafact zifat/Productos_Zifact_Migrado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Productos" sheetId="1" r:id="rId1"/>
+    <sheet name="Plantilla" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -406,22 +406,22 @@
         <v>Nombre</v>
       </c>
       <c r="B1" t="str">
-        <v>Código Principal</v>
+        <v>Codigo Principal</v>
       </c>
       <c r="C1" t="str">
-        <v>Código Auxiliar</v>
+        <v>Codigo Auxiliar</v>
       </c>
       <c r="D1" t="str">
         <v>Precio Unitario</v>
       </c>
       <c r="E1" t="str">
-        <v>Código IVA</v>
+        <v>Codigo IVA</v>
       </c>
       <c r="F1" t="str">
-        <v>Código ICE</v>
+        <v>Codigo ICE</v>
       </c>
       <c r="G1" t="str">
-        <v>Código IRBPNR</v>
+        <v>Codigo IRBPNR</v>
       </c>
       <c r="H1" t="str">
         <v>Estado (A/I)</v>

</xml_diff>